<commit_message>
minor code refactors to step 5
</commit_message>
<xml_diff>
--- a/tables/hlm-tables.xlsx
+++ b/tables/hlm-tables.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nnapo\Documents\PhD Classes\Tesis 1-6\analysis\thesis-analysis\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70164688-8F13-4ABC-B79D-B422819FDB23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DA38A5-7A54-4A45-A305-C955B3596831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tbl20" sheetId="2" r:id="rId1"/>
     <sheet name="tbl21" sheetId="1" r:id="rId2"/>
+    <sheet name="tbl22" sheetId="3" r:id="rId3"/>
+    <sheet name="tbl23" sheetId="4" r:id="rId4"/>
+    <sheet name="tbl24" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="39">
   <si>
     <t>Parameter</t>
   </si>
@@ -103,32 +106,6 @@
     <t>0.001 **</t>
   </si>
   <si>
-    <r>
-      <t>Table 21</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Two-Level Model Results for H&amp;F Overall (Inhibitory Control)</t>
-    </r>
-  </si>
-  <si>
     <t>&lt;.001***</t>
   </si>
   <si>
@@ -142,6 +119,33 @@
   </si>
   <si>
     <t>0.001**</t>
+  </si>
+  <si>
+    <t>corsi</t>
+  </si>
+  <si>
+    <t>hnf</t>
+  </si>
+  <si>
+    <t>dccs</t>
+  </si>
+  <si>
+    <t>.002**</t>
+  </si>
+  <si>
+    <t>.018*</t>
+  </si>
+  <si>
+    <t>woodcock-munoz</t>
+  </si>
+  <si>
+    <t>.024*</t>
+  </si>
+  <si>
+    <t>tejasLee</t>
+  </si>
+  <si>
+    <t>&lt;.001</t>
   </si>
 </sst>
 </file>
@@ -151,7 +155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,14 +171,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -507,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84C52E79-E91E-4EA7-BF15-5154CA34C86E}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.90625" bestFit="1" customWidth="1"/>
@@ -856,6 +852,11 @@
       </c>
       <c r="F17" s="2">
         <v>0.17799999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -913,7 +914,7 @@
         <v>25.85</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -933,7 +934,7 @@
         <v>-2.16</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -993,7 +994,7 @@
         <v>2.0299999999999998</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -1013,7 +1014,7 @@
         <v>-8.1999999999999993</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -1033,7 +1034,7 @@
         <v>3.44</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -1053,7 +1054,7 @@
         <v>2.44</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -1093,7 +1094,7 @@
         <v>3.3</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
@@ -1217,8 +1218,11 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="5" t="s">
-        <v>25</v>
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
@@ -1428,4 +1432,1715 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93FAE91C-26BF-44EB-A4A7-84C5365E4446}">
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="34.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3">
+        <v>6.86</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="D2" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E2" s="3">
+        <v>27.21</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="D3" s="3">
+        <v>177</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0.23</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.34</v>
+      </c>
+      <c r="D4" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.67</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.504</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3">
+        <v>-0.2</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.36</v>
+      </c>
+      <c r="D5" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E5" s="3">
+        <v>-0.55000000000000004</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.58099999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0.17</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.33</v>
+      </c>
+      <c r="D6" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.51</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3">
+        <v>-1.4</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0.32</v>
+      </c>
+      <c r="D7" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E7" s="3">
+        <v>-4.32</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.38</v>
+      </c>
+      <c r="D8" s="3">
+        <v>177</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.78</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.437</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3">
+        <v>1.29</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0.41</v>
+      </c>
+      <c r="D9" s="3">
+        <v>177</v>
+      </c>
+      <c r="E9" s="3">
+        <v>3.14</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3">
+        <v>0.44</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0.37</v>
+      </c>
+      <c r="D10" s="3">
+        <v>177</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.23300000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="3">
+        <v>-0.18</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0.37</v>
+      </c>
+      <c r="D11" s="3">
+        <v>177</v>
+      </c>
+      <c r="E11" s="3">
+        <v>-0.48</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="3">
+        <v>-0.63</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.47</v>
+      </c>
+      <c r="D12" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E12" s="3">
+        <v>-1.35</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.17699999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="3">
+        <v>0.18</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0.47</v>
+      </c>
+      <c r="D13" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E13" s="3">
+        <v>0.39</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.69899999999999995</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0.21</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0.48</v>
+      </c>
+      <c r="D14" s="3">
+        <v>313.83999999999997</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0.43</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.66600000000000004</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="3">
+        <v>1.27</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.53</v>
+      </c>
+      <c r="D15" s="3">
+        <v>177</v>
+      </c>
+      <c r="E15" s="3">
+        <v>2.39</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="3">
+        <v>-0.79</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.54</v>
+      </c>
+      <c r="D16" s="3">
+        <v>177</v>
+      </c>
+      <c r="E16" s="3">
+        <v>-1.47</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.14299999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="3">
+        <v>-0.18</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.54</v>
+      </c>
+      <c r="D17" s="3">
+        <v>177</v>
+      </c>
+      <c r="E17" s="3">
+        <v>-0.33</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.74099999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="7"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="7"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="6"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="6"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="6"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="6"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="6"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="6"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="6"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="6"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="6"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="6"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="6"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="6"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="6"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="6"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="6"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="6"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="7"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="6"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="6"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="7"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="6"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="6"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="6"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="6"/>
+      <c r="B46" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E9EFAA9-6389-4BAD-B3F4-0D03E9FBE751}">
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="34.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3">
+        <v>64.45</v>
+      </c>
+      <c r="C2" s="3">
+        <v>2.09</v>
+      </c>
+      <c r="D2" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E2" s="3">
+        <v>30.88</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1.72</v>
+      </c>
+      <c r="D3" s="3">
+        <v>177</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.58099999999999996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2.59</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="D4" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.93</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.35599999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3">
+        <v>-0.24</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="D5" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E5" s="3">
+        <v>-0.08</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.93600000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1.18</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2.69</v>
+      </c>
+      <c r="D6" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.44</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.66100000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3">
+        <v>-18.68</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2.68</v>
+      </c>
+      <c r="D7" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E7" s="3">
+        <v>-6.98</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="3">
+        <v>0.41</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D8" s="3">
+        <v>177</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0.18</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.85899999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C9" s="3">
+        <v>2.46</v>
+      </c>
+      <c r="D9" s="3">
+        <v>177</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.25900000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3">
+        <v>1.28</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="D10" s="3">
+        <v>177</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.56299999999999994</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="3">
+        <v>2.66</v>
+      </c>
+      <c r="C11" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D11" s="3">
+        <v>177</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1.21</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0.22800000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="3">
+        <v>-3.51</v>
+      </c>
+      <c r="C12" s="3">
+        <v>3.87</v>
+      </c>
+      <c r="D12" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E12" s="3">
+        <v>-0.91</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.36499999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="3">
+        <v>-8.91</v>
+      </c>
+      <c r="C13" s="3">
+        <v>3.92</v>
+      </c>
+      <c r="D13" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E13" s="3">
+        <v>-2.27</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="3">
+        <v>-6.52</v>
+      </c>
+      <c r="C14" s="3">
+        <v>3.94</v>
+      </c>
+      <c r="D14" s="3">
+        <v>246.16</v>
+      </c>
+      <c r="E14" s="3">
+        <v>-1.66</v>
+      </c>
+      <c r="F14" s="4">
+        <v>9.9000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="3">
+        <v>3.83</v>
+      </c>
+      <c r="C15" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="D15" s="3">
+        <v>177</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0.23100000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="3">
+        <v>1.89</v>
+      </c>
+      <c r="C16" s="3">
+        <v>3.23</v>
+      </c>
+      <c r="D16" s="3">
+        <v>177</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0.59</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.55800000000000005</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="3">
+        <v>7.35</v>
+      </c>
+      <c r="C17" s="3">
+        <v>3.24</v>
+      </c>
+      <c r="D17" s="3">
+        <v>177</v>
+      </c>
+      <c r="E17" s="3">
+        <v>2.27</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="7"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="7"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="6"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="6"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="6"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="6"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="6"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="6"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="6"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="6"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="6"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="6"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="6"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="6"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="6"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="6"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="6"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="6"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="7"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="6"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="6"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="7"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="6"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="6"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="6"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="6"/>
+      <c r="B46" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA238E7A-6BC6-4496-80FB-EFC2AFA64233}">
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="34.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3">
+        <v>63.55</v>
+      </c>
+      <c r="C2" s="3">
+        <v>2.39</v>
+      </c>
+      <c r="D2" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E2" s="3">
+        <v>26.62</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1.75</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1.79</v>
+      </c>
+      <c r="D3" s="3">
+        <v>177</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.98</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.32900000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0.13</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="D4" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.96799999999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3">
+        <v>-1.1299999999999999</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.42</v>
+      </c>
+      <c r="D5" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E5" s="3">
+        <v>-0.33</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.74199999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3.08</v>
+      </c>
+      <c r="D6" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.35</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.72599999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3">
+        <v>-27.71</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.06</v>
+      </c>
+      <c r="D7" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E7" s="3">
+        <v>-9.0500000000000007</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="3">
+        <v>3.05</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="D8" s="3">
+        <v>177</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1.27</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.20499999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3">
+        <v>2.46</v>
+      </c>
+      <c r="C9" s="3">
+        <v>2.56</v>
+      </c>
+      <c r="D9" s="3">
+        <v>177</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0.96</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.33800000000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3">
+        <v>1.78</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2.31</v>
+      </c>
+      <c r="D10" s="3">
+        <v>177</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0.77</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="3">
+        <v>3.48</v>
+      </c>
+      <c r="C11" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="D11" s="3">
+        <v>177</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1.52</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0.13100000000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="3">
+        <v>-2.82</v>
+      </c>
+      <c r="C12" s="3">
+        <v>4.43</v>
+      </c>
+      <c r="D12" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E12" s="3">
+        <v>-0.64</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.52500000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="3">
+        <v>-3.63</v>
+      </c>
+      <c r="C13" s="3">
+        <v>4.49</v>
+      </c>
+      <c r="D13" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E13" s="3">
+        <v>-0.81</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="3">
+        <v>-0.42</v>
+      </c>
+      <c r="C14" s="3">
+        <v>4.51</v>
+      </c>
+      <c r="D14" s="3">
+        <v>233.13</v>
+      </c>
+      <c r="E14" s="3">
+        <v>-0.09</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.92500000000000004</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="3">
+        <v>1.72</v>
+      </c>
+      <c r="C15" s="3">
+        <v>3.32</v>
+      </c>
+      <c r="D15" s="3">
+        <v>177</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.52</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0.60399999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="3">
+        <v>2.65</v>
+      </c>
+      <c r="C16" s="3">
+        <v>3.36</v>
+      </c>
+      <c r="D16" s="3">
+        <v>177</v>
+      </c>
+      <c r="E16" s="3">
+        <v>0.79</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.432</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="3">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="C17" s="3">
+        <v>3.37</v>
+      </c>
+      <c r="D17" s="3">
+        <v>177</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0.72</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.47199999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="7"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="7"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="6"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="6"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="6"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="6"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="6"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="6"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="6"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="6"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="6"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="6"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="6"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="6"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="6"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="6"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="6"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="6"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="7"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="6"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="6"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="7"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="6"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="6"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="6"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="6"/>
+      <c r="B46" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>